<commit_message>
Ajout PE Waterfall européen Fund Beta (deal MedTech Solutions) - étape 5a
</commit_message>
<xml_diff>
--- a/beta/fund_beta_waterfall.xlsx
+++ b/beta/fund_beta_waterfall.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\devil\fund accounting roadmap\lux-fund-case-study\beta\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5F3DECDB-DA67-43BB-ACBC-E3785EF3DA4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{9564D62F-CFA8-4764-8C55-DE935241A978}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{183BB934-16D1-4881-812E-63FEED958496}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="37">
   <si>
     <t>Legal Structure</t>
   </si>
@@ -129,6 +129,30 @@
   </si>
   <si>
     <t>Catch-Up Amount</t>
+  </si>
+  <si>
+    <t>Stage 4 — Carried Interest</t>
+  </si>
+  <si>
+    <t>LP Share</t>
+  </si>
+  <si>
+    <t>GP Share</t>
+  </si>
+  <si>
+    <t>VERIFICATION</t>
+  </si>
+  <si>
+    <t>Total LP</t>
+  </si>
+  <si>
+    <t>Total GP</t>
+  </si>
+  <si>
+    <t>Total Distributed</t>
+  </si>
+  <si>
+    <t>GP % of Total Profit</t>
   </si>
 </sst>
 </file>
@@ -204,7 +228,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -228,6 +252,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Milliers" xfId="1" builtinId="3"/>
@@ -688,14 +715,14 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7CF0810-BA3A-4340-AAA9-371451B485B2}">
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="10" t="s">
         <v>16</v>
       </c>
@@ -703,7 +730,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
         <v>18</v>
       </c>
@@ -711,7 +738,7 @@
         <v>8000000</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
         <v>19</v>
       </c>
@@ -719,7 +746,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="10" t="s">
         <v>20</v>
       </c>
@@ -727,7 +754,7 @@
         <v>16500000</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
         <v>21</v>
       </c>
@@ -736,12 +763,12 @@
         <v>16500000</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="10" t="s">
         <v>23</v>
       </c>
@@ -750,7 +777,7 @@
         <v>8000000</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="10" t="s">
         <v>24</v>
       </c>
@@ -759,20 +786,21 @@
         <v>8500000</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="10" t="s">
         <v>5</v>
       </c>
       <c r="B12" s="4">
         <v>0.08</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="F12" s="1"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="10" t="s">
         <v>26</v>
       </c>
@@ -781,7 +809,7 @@
         <v>2883911.6800000025</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="10" t="s">
         <v>24</v>
       </c>
@@ -790,7 +818,7 @@
         <v>5616088.3199999975</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="11" t="s">
         <v>27</v>
       </c>
@@ -800,8 +828,8 @@
         <v>28</v>
       </c>
       <c r="B17" s="2">
-        <f>+B13*'Fund Identity'!B7</f>
-        <v>576782.33600000048</v>
+        <f>+B13*25%</f>
+        <v>720977.92000000062</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
@@ -810,7 +838,71 @@
       </c>
       <c r="B18" s="12">
         <f>+B14-B17</f>
-        <v>5039305.9839999974</v>
+        <v>4895110.3999999966</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" s="13" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="B21" s="2">
+        <f>+B18*0.8</f>
+        <v>3916088.3199999975</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="B22" s="2">
+        <f>+B18*0.2</f>
+        <v>979022.07999999938</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A25" s="13" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A26" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="B26" s="3">
+        <f>+B21+B13+B8</f>
+        <v>14800000</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A27" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="B27" s="3">
+        <f>+B17+B22</f>
+        <v>1700000</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A28" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="B28" s="3">
+        <f>+B22+B21+B17+B13+B8</f>
+        <v>16500000</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A29" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="B29" s="3">
+        <f>+B27/(B28-B2)</f>
+        <v>0.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>